<commit_message>
Qualify the proof-of-origin wording in the shipment notes
The note asserted that the modernised EU-Mexico agreement replaces EUR.1
and the invoice declaration with a REX statement on origin. That came
from secondary trade press, not a primary source, and which regime
applies at the clearance date was not verified.

Now names both forms and marks the form of proof as to be confirmed. The
underlying finding is unchanged: no proof of preferential origin in any
form is present in the documents, so the 5% third-country rate applies.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dm8VBjzptt4ipwDaF6pt1X
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Strand_Cosmetics_Europe_HBL875606112905.xlsx
+++ b/output/HS_Code_Summary_Strand_Cosmetics_Europe_HBL875606112905.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="156">
   <si>
     <t xml:space="preserve">Odesílatel (sender)</t>
   </si>
@@ -167,16 +167,22 @@
     <t xml:space="preserve">Skutečný rozdíl bude vyšší – celní hodnota se navýší o dopravu do Hamburku.</t>
   </si>
   <si>
-    <t xml:space="preserve">→ DOPORUČENÍ: vyžádat od Vitro Envases SA de CV prohlášení o preferenčním původu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   (u modernizované Globální dohody EU–Mexiko se používá prohlášení o původu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   registrovaného vývozce v systému REX; dříve EUR.1 / fakturační prohlášení)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   PŘED podáním celního prohlášení, případně požádat o dodatečné vrácení cla.</t>
+    <t xml:space="preserve">→ DOPORUČENÍ: vyžádat od Vitro Envases SA de CV preferenční důkaz původu PŘED podáním</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   celního prohlášení, případně následně požádat o dodatečné vrácení cla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Formu důkazu OVĚŘIT k datu propuštění: dle Globální dohody EU–Mexiko (rozhodnutí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   2/2000) je to EUR.1 nebo fakturační prohlášení; modernizovaná dohoda má tyto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   doklady nahradit prohlášením o původu registrovaného vývozce (REX).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Neověřeno u primárního zdroje – potvrdit s celní správou / u dovozce.</t>
   </si>
   <si>
     <t xml:space="preserve">▌ DODANÉ DOKUMENTY (stav 3.8.2026)</t>
@@ -1258,7 +1264,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A88"/>
+  <dimension ref="A1:A90"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="125"/>
@@ -1331,20 +1337,20 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11"/>
+      <c r="A15" s="11" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
-        <v>51</v>
+      <c r="A16" s="11" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>52</v>
-      </c>
+      <c r="A17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="16" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1359,20 +1365,20 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11"/>
+      <c r="A21" s="11" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>56</v>
+      <c r="A22" s="11" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>57</v>
-      </c>
+      <c r="A23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="17" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1397,20 +1403,20 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11"/>
+      <c r="A29" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="s">
-        <v>63</v>
+      <c r="A30" s="11" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>64</v>
-      </c>
+      <c r="A31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="16" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1435,17 +1441,17 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11"/>
+      <c r="A37" s="11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>71</v>
-      </c>
+      <c r="A39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
@@ -1478,17 +1484,17 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11"/>
+      <c r="A46" s="11" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11" t="s">
-        <v>79</v>
-      </c>
+      <c r="A48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
@@ -1511,26 +1517,26 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11"/>
+      <c r="A53" s="11" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="16" t="s">
-        <v>84</v>
+      <c r="A54" s="11" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="11" t="s">
-        <v>19</v>
-      </c>
+      <c r="A55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11" t="s">
-        <v>85</v>
+      <c r="A56" s="16" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1539,20 +1545,20 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11"/>
+      <c r="A59" s="11" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="16" t="s">
-        <v>88</v>
+      <c r="A60" s="11" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="11" t="s">
-        <v>89</v>
-      </c>
+      <c r="A61" s="11"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="16" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1582,43 +1588,43 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="17" t="s">
+      <c r="A68" s="11" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="11"/>
+      <c r="A69" s="11" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="16" t="s">
-        <v>97</v>
+      <c r="A70" s="17" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="11" t="s">
-        <v>98</v>
-      </c>
+      <c r="A71" s="11"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="11" t="s">
+      <c r="A72" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="11"/>
+      <c r="A73" s="11" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="16" t="s">
-        <v>100</v>
+      <c r="A74" s="11" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="11" t="s">
-        <v>101</v>
-      </c>
+      <c r="A75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="16" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1628,20 +1634,20 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="11"/>
+      <c r="A78" s="11" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="16" t="s">
-        <v>104</v>
+      <c r="A79" s="11" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="11" t="s">
-        <v>105</v>
-      </c>
+      <c r="A80" s="11"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="11" t="s">
+      <c r="A81" s="16" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1661,21 +1667,31 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="11"/>
+      <c r="A85" s="11" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="16" t="s">
-        <v>110</v>
+      <c r="A86" s="11" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="11" t="s">
-        <v>111</v>
-      </c>
+      <c r="A87" s="11"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="11" t="s">
+      <c r="A88" s="16" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="11" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1705,269 +1721,269 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>31040</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">B5+B6+B7</f>
         <v>31040</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B10" s="23" t="n">
         <v>0.05</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">B8*B10</f>
         <v>1552</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B12" s="24" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">B8*B12</f>
         <v>0</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">B11*B12</f>
         <v>0</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B16" s="21" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">B13+B14+B16</f>
         <v>0</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B18" s="23" t="n">
         <v>0.21</v>
       </c>
       <c r="C18" s="11"/>
       <c r="D18" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">B17*B18</f>
         <v>0</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B22" s="23" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="11"/>
       <c r="D22" s="12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B23" s="22" t="n">
         <f aca="false">B8*B22</f>
         <v>0</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B24" s="25" t="n">
         <f aca="false">B11-B23</f>
         <v>1552</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B25" s="25" t="n">
         <f aca="false">B24*B12</f>
         <v>0</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>